<commit_message>
publish: 2026-02-24 12:57 GMT
</commit_message>
<xml_diff>
--- a/files/Downloads/Week 7/Regression_Calculations_Week 7.xlsx
+++ b/files/Downloads/Week 7/Regression_Calculations_Week 7.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10215"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livewarwickac-my.sharepoint.com/personal/u1373867_live_warwick_ac_uk/Documents/Warwick/Modules/PO12Q/Seminars/PO12Q_Seminar_Week 7/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u1373867/Dropbox/PO12Q/files/Downloads/Week 7/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="244" documentId="11_144A03E2ACE44B6A332A7933CA070F099E6AD964" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B2B627D-A81D-7745-9D77-7EB3AE970B69}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD2D12E2-2FB4-C44B-AF30-F1F7788A8227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="940" yWindow="500" windowWidth="27820" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="960" yWindow="660" windowWidth="27820" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -287,7 +287,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -327,8 +327,8 @@
       <xdr:rowOff>14763</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="188065" cy="175369"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="TextBox 1">
@@ -423,7 +423,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="TextBox 1">
@@ -498,8 +498,8 @@
       <xdr:rowOff>8467</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="117853" cy="172227"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="TextBox 2">
@@ -573,7 +573,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="TextBox 2">
@@ -641,8 +641,8 @@
       <xdr:rowOff>6296</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="429092" cy="184987"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="TextBox 3">
@@ -771,7 +771,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="TextBox 3">
@@ -839,8 +839,8 @@
       <xdr:rowOff>198801</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="425822" cy="184987"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="TextBox 4">
@@ -969,7 +969,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="TextBox 4">
@@ -1037,8 +1037,8 @@
       <xdr:rowOff>23452</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="583467" cy="175369"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="TextBox 5">
@@ -1080,6 +1080,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1119,7 +1120,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="TextBox 5">
@@ -1189,8 +1190,8 @@
       <xdr:rowOff>20721</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="424795" cy="172227"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="TextBox 6">
@@ -1232,6 +1233,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1276,7 +1278,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="TextBox 6">
@@ -1340,8 +1342,8 @@
       <xdr:rowOff>14036</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="545214" cy="175369"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="TextBox 7">
@@ -1383,6 +1385,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1458,7 +1461,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="TextBox 7">
@@ -1528,8 +1531,8 @@
       <xdr:rowOff>20054</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="307969" cy="172227"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="TextBox 8">
@@ -1608,7 +1611,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="TextBox 8">
@@ -1676,8 +1679,8 @@
       <xdr:rowOff>20052</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="541237" cy="175369"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="10" name="TextBox 9">
@@ -1719,6 +1722,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1794,7 +1798,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="10" name="TextBox 9">
@@ -1864,8 +1868,8 @@
       <xdr:rowOff>6016</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1047916" cy="172227"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="11" name="TextBox 10">
@@ -1907,6 +1911,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1953,13 +1958,7 @@
                       <a:rPr lang="en-US" sz="1100" b="0" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                       </a:rPr>
-                      <m:t>)</m:t>
-                    </m:r>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>(</m:t>
+                      <m:t>)(</m:t>
                     </m:r>
                     <m:r>
                       <a:rPr lang="en-US" sz="1100" b="0" i="1">
@@ -2005,7 +2004,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="11" name="TextBox 10">
@@ -2069,8 +2068,8 @@
       <xdr:rowOff>7352</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="337280" cy="172227"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="TextBox 11">
@@ -2112,6 +2111,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2144,7 +2144,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="TextBox 11">
@@ -2208,8 +2208,8 @@
       <xdr:rowOff>6684</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="434474" cy="172227"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="13" name="TextBox 12">
@@ -2251,6 +2251,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2307,7 +2308,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="13" name="TextBox 12">
@@ -2371,8 +2372,8 @@
       <xdr:rowOff>14037</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="607282" cy="175369"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="14" name="TextBox 13">
@@ -2414,6 +2415,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2501,7 +2503,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="14" name="TextBox 13">
@@ -2571,8 +2573,8 @@
       <xdr:rowOff>6684</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="434474" cy="172227"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="15" name="TextBox 14">
@@ -2614,6 +2616,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2664,7 +2667,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="15" name="TextBox 14">
@@ -2728,8 +2731,8 @@
       <xdr:rowOff>14037</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="607281" cy="175304"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="16" name="TextBox 15">
@@ -2771,6 +2774,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2846,7 +2850,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="16" name="TextBox 15">
@@ -2916,8 +2920,8 @@
       <xdr:rowOff>26736</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="176464" cy="173789"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="17" name="TextBox 16">
@@ -2959,6 +2963,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2998,7 +3003,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="17" name="TextBox 16">
@@ -4054,15 +4059,15 @@
     <row r="20" spans="11:14" x14ac:dyDescent="0.2">
       <c r="M20" s="12"/>
       <c r="N20" s="16">
-        <f>N18/G14^0.5</f>
-        <v>7.3248270698394933</v>
+        <f>(N14/(10*G14))^0.5*N18</f>
+        <v>304.71632763644988</v>
       </c>
     </row>
     <row r="21" spans="11:14" x14ac:dyDescent="0.2">
       <c r="M21" s="14"/>
       <c r="N21" s="17">
-        <f>(N14/(10*G14))^0.5*N18</f>
-        <v>304.71632763644988</v>
+        <f>N18/G14^0.5</f>
+        <v>7.3248270698394933</v>
       </c>
     </row>
   </sheetData>

</xml_diff>